<commit_message>
:skunk:CCA calculations with final data
</commit_message>
<xml_diff>
--- a/data/derived_data/6_NMI_CCA/Dataset_2/CCA_CONFIGS_ITS_D2.xlsx
+++ b/data/derived_data/6_NMI_CCA/Dataset_2/CCA_CONFIGS_ITS_D2.xlsx
@@ -422,10 +422,10 @@
         <v>18.8227462005675</v>
       </c>
       <c r="E2" t="n">
-        <v>0.001</v>
+        <v>0.0002</v>
       </c>
       <c r="F2" t="n">
-        <v>0.076</v>
+        <v>0.016</v>
       </c>
     </row>
     <row r="3">
@@ -442,10 +442,10 @@
         <v>12.9622303502903</v>
       </c>
       <c r="E3" t="n">
-        <v>0.001</v>
+        <v>0.0002</v>
       </c>
       <c r="F3" t="n">
-        <v>0.015</v>
+        <v>0.00919999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -462,10 +462,10 @@
         <v>13.8634485749429</v>
       </c>
       <c r="E4" t="n">
-        <v>0.001</v>
+        <v>0.0002</v>
       </c>
       <c r="F4" t="n">
-        <v>0.022</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="5">
@@ -482,10 +482,10 @@
         <v>8.55583080840544</v>
       </c>
       <c r="E5" t="n">
-        <v>0.001</v>
+        <v>0.0002</v>
       </c>
       <c r="F5" t="n">
-        <v>0.032</v>
+        <v>0.000800000000000023</v>
       </c>
     </row>
     <row r="6">
@@ -502,7 +502,7 @@
         <v>8.00800590138213</v>
       </c>
       <c r="E6" t="n">
-        <v>0.001</v>
+        <v>0.0002</v>
       </c>
       <c r="F6" t="n">
         <v>0.00600000000000001</v>

</xml_diff>